<commit_message>
feat: keep name, brand, and model in separate columns
Excel import template now includes brand/model columns with instructions not to fold them into the product name. Quotes, invoices, and print tables show name, brand, and model as their own columns instead of stacking details under the name.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/frontend/public/templates/products-import-template.xlsx
+++ b/frontend/public/templates/products-import-template.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="31">
   <si>
     <t>اسم الصنف</t>
   </si>
@@ -30,6 +30,12 @@
     <t>الباركود</t>
   </si>
   <si>
+    <t>الماركة</t>
+  </si>
+  <si>
+    <t>الموديل</t>
+  </si>
+  <si>
     <t>سعر التكلفة</t>
   </si>
   <si>
@@ -57,6 +63,12 @@
     <t>قطعة</t>
   </si>
   <si>
+    <t>سامسونج</t>
+  </si>
+  <si>
+    <t>A54</t>
+  </si>
+  <si>
     <t>المخزن الرئيسي</t>
   </si>
   <si>
@@ -66,22 +78,28 @@
     <t>الشرح</t>
   </si>
   <si>
-    <t>مطلوب</t>
-  </si>
-  <si>
-    <t>اختياري — اسم التصنيف الموجود في النظام</t>
-  </si>
-  <si>
-    <t>اختياري — اسم وحدة القياس الموجودة في النظام</t>
+    <t>مطلوب — اسم الصنف فقط، بدون الماركة أو الموديل</t>
+  </si>
+  <si>
+    <t>اختياري — إن لم يوجد يُنشأ تلقائياً بالاسم المكتوب</t>
+  </si>
+  <si>
+    <t>اختياري — إن فرغت تُستخدم «قطعة»؛ وإن لم توجد تُنشأ تلقائياً</t>
   </si>
   <si>
     <t>اختياري — يجب أن يكون فريداً إن وُجد</t>
   </si>
   <si>
+    <t>اختياري — عمود مستقل، لا تضعها داخل اسم الصنف</t>
+  </si>
+  <si>
+    <t>اختياري — عمود مستقل، لا تضعه داخل اسم الصنف</t>
+  </si>
+  <si>
     <t>اختياري — افتراضي 0</t>
   </si>
   <si>
-    <t>مطلوب — اسم أو رمز المخزن لربط الصنف</t>
+    <t>مطلوب — اسم أو رمز مخزن موجود. إن لم يكن لديك أي مخزن يُنشأ «المخزن الرئيسي» تلقائياً</t>
   </si>
   <si>
     <t>اختياري — تُحفظ في وصف الصنف</t>
@@ -448,22 +466,24 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="12.854" bestFit="true" customWidth="true" style="0"/>
     <col min="2" max="2" width="9.283" bestFit="true" customWidth="true" style="0"/>
     <col min="3" max="3" width="8.141" bestFit="true" customWidth="true" style="0"/>
     <col min="4" max="4" width="10.569" bestFit="true" customWidth="true" style="0"/>
-    <col min="5" max="5" width="13.997" bestFit="true" customWidth="true" style="0"/>
-    <col min="6" max="6" width="11.711" bestFit="true" customWidth="true" style="0"/>
-    <col min="7" max="7" width="17.567" bestFit="true" customWidth="true" style="0"/>
-    <col min="8" max="8" width="16.425" bestFit="true" customWidth="true" style="0"/>
+    <col min="5" max="5" width="9.283" bestFit="true" customWidth="true" style="0"/>
+    <col min="6" max="6" width="9.283" bestFit="true" customWidth="true" style="0"/>
+    <col min="7" max="7" width="13.997" bestFit="true" customWidth="true" style="0"/>
+    <col min="8" max="8" width="11.711" bestFit="true" customWidth="true" style="0"/>
     <col min="9" max="9" width="17.567" bestFit="true" customWidth="true" style="0"/>
-    <col min="10" max="10" width="9.283" bestFit="true" customWidth="true" style="0"/>
+    <col min="10" max="10" width="16.425" bestFit="true" customWidth="true" style="0"/>
+    <col min="11" max="11" width="17.567" bestFit="true" customWidth="true" style="0"/>
+    <col min="12" max="12" width="9.283" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -494,30 +514,42 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:10">
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
       <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2">
         <v>10</v>
       </c>
-      <c r="B2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2">
-        <v>10</v>
-      </c>
-      <c r="F2">
+      <c r="H2">
         <v>15</v>
       </c>
-      <c r="G2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2">
+      <c r="I2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2">
         <v>0</v>
       </c>
-      <c r="I2">
+      <c r="K2">
         <v>5</v>
       </c>
     </row>
@@ -533,19 +565,19 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="18.71" bestFit="true" customWidth="true" style="0"/>
-    <col min="2" max="2" width="52.987" bestFit="true" customWidth="true" style="0"/>
+    <col min="2" max="2" width="101.404" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -553,7 +585,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -561,7 +593,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -569,7 +601,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -577,7 +609,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -585,7 +617,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -593,7 +625,7 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -601,7 +633,7 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -609,7 +641,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -617,7 +649,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -625,15 +657,31 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>24</v>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" t="s">
+        <v>29</v>
+      </c>
+      <c r="B14" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>